<commit_message>
tag 4 and internal notes
</commit_message>
<xml_diff>
--- a/SFO_Technologies/Default Item.xlsx
+++ b/SFO_Technologies/Default Item.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191028" fullCalcOnLoad="1"/>
@@ -449,7 +449,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL4"/>
+  <dimension ref="A1:AN4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="12" max="12"/>
@@ -521,130 +521,140 @@
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Not visible to vendors.</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
           <t>The name of a specification (e.g. color, manufacturor, weight, density) associated with this item</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>The required value for the specification in the previous column</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>The required measurement unit for the specification in the previous column</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>The name of a specification (e.g. color, manufacturor, weight, density) associated with this item</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>The required value for the specification in the previous column</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>The required measurement unit for the specification in the previous column</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>The name of a specification (e.g. color, manufacturor, weight, density) associated with this item</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>The required value for the specification in the previous column</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>The required measurement unit for the specification in the previous column</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Universal or internal identifier name for this item (e.g. SKU id, UCAS ID, pubchem ID)</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Value associated with identifier in previous column</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Choice TRUE: The entity is a buyer of the item; FALSE: The entity is not a buyer of the item</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>The currency in which the entity buys the item (e.g.: INR, USD, JPY)</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>The price in which the entity buys the item</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>Choice TRUE: The entity is a seller of the item; FALSE: The entity is not a seller of the item</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>Tag to group this item by</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>Tag to group this item by</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>Tag to group this item by</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Tag to group this item by</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
         <is>
           <t>The item's depth in the BOM hierarchy; 1 is a direct child of the finished good. Used to build the BOM file, not imported with the item.</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>How much of this item the parent assembly consumes. Used to build the BOM file, not imported with the item.</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>The quantity this BOM is defined for. Used to build the BOM file, not imported with the item.</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>The name of the entity which procures this item. The settings after this column will apply for this entity only. An item can only be procured by entities to which it is linked. If multiple entities procure this item, then add more rows. The new rows can have different entity names and setings, but all the item details (to the left of this column) should be identical.</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>Preferred vendors are highlighted when procuring items. It is recommended to include at least one preferred vendor per item. Vendor codes can be downloaded from the vendor directory of FactWise Admin if you do not have them handy. You can insert more columns named 'Preferred vendor code' to include multiple preferred vendors for an item</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>Add an alternate, vendor-specific name for the item that applies only to the selected vendor</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>Preferred vendors are highlighted when procuring items. It is recommended to include at least one preferred vendor per item. Vendor codes can be downloaded from the vendor directory of FactWise Admin if you do not have them handy. You can insert more columns named 'Preferred vendor code' to include multiple preferred vendors for an item</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>Add an alternate, vendor-specific name for the item that applies only to the selected vendor</t>
         </is>
@@ -713,130 +723,140 @@
       </c>
       <c r="M2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Optional, </t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
           <t>Optional, Max 100 characters e.g. 'Color'</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters. If multiple options are fine, provide a list separated with '/' e.g. 'Blue / Green'</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>Optional, measurement unit names or abbreviations. e.g. 'kg, gm, units'</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters e.g. 'Color'</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters. If multiple options are fine, provide a list separated with '/' e.g. 'Blue / Green'</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Optional, measurement unit names or abbreviations. e.g. 'kg, gm, units'</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="T2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters e.g. 'Color'</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters. If multiple options are fine, provide a list separated with '/' e.g. 'Blue / Green'</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>Optional, measurement unit names or abbreviations. e.g. 'kg, gm, units'</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="W2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters e.g. UCAS ID</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters e.g. 123-456-7890</t>
         </is>
       </c>
-      <c r="X2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t xml:space="preserve">Optional, </t>
         </is>
       </c>
-      <c r="Y2" t="inlineStr">
+      <c r="Z2" t="inlineStr">
         <is>
           <t xml:space="preserve">Optional, </t>
         </is>
       </c>
-      <c r="Z2" t="inlineStr">
+      <c r="AA2" t="inlineStr">
         <is>
           <t xml:space="preserve">Optional, </t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
+      <c r="AB2" t="inlineStr">
         <is>
           <t xml:space="preserve">Optional, </t>
         </is>
       </c>
-      <c r="AB2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>Optional, Max 30 characters</t>
         </is>
       </c>
-      <c r="AC2" t="inlineStr">
+      <c r="AD2" t="inlineStr">
         <is>
           <t>Optional, Max 30 characters</t>
         </is>
       </c>
-      <c r="AD2" t="inlineStr">
+      <c r="AE2" t="inlineStr">
         <is>
           <t>Optional, Max 30 characters</t>
         </is>
       </c>
-      <c r="AE2" t="inlineStr">
+      <c r="AF2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Optional, </t>
+        </is>
+      </c>
+      <c r="AG2" t="inlineStr">
         <is>
           <t>Optional, whole number</t>
         </is>
       </c>
-      <c r="AF2" t="inlineStr">
+      <c r="AH2" t="inlineStr">
         <is>
           <t>Optional, number, zero allowed</t>
         </is>
       </c>
-      <c r="AG2" t="inlineStr">
+      <c r="AI2" t="inlineStr">
         <is>
           <t>Optional, number greater than zero</t>
         </is>
       </c>
-      <c r="AH2" t="inlineStr">
+      <c r="AJ2" t="inlineStr">
         <is>
           <t>Required, Name of an entity which should be able to procure this item. The entity should belong to the enterprise the current user belongs to</t>
         </is>
       </c>
-      <c r="AI2" t="inlineStr">
+      <c r="AK2" t="inlineStr">
         <is>
           <t>Optional, Vendor code of preferred vendor for this item. The vendor code should exist for the enterprise the current user belongs toe.g. 'V001'</t>
         </is>
       </c>
-      <c r="AJ2" t="inlineStr">
+      <c r="AL2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters</t>
         </is>
       </c>
-      <c r="AK2" t="inlineStr">
+      <c r="AM2" t="inlineStr">
         <is>
           <t>Optional, Vendor code of preferred vendor for this item. The vendor code should exist for the enterprise the current user belongs toe.g. 'V001'</t>
         </is>
       </c>
-      <c r="AL2" t="inlineStr">
+      <c r="AN2" t="inlineStr">
         <is>
           <t>Optional, Max 100 characters</t>
         </is>
@@ -845,7 +865,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve"> </t>
         </is>
       </c>
     </row>
@@ -907,135 +927,145 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
+          <t>Internal notes</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
           <t>SAP Description</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Specification name (1)</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="O4" t="inlineStr">
         <is>
           <t>Specification value (1)</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
+      <c r="P4" t="inlineStr">
         <is>
           <t>Specification UOM (1)</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
+      <c r="Q4" t="inlineStr">
         <is>
           <t>Specification name (2)</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>Specification value (2)</t>
         </is>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Specification UOM (2)</t>
         </is>
       </c>
-      <c r="S4" t="inlineStr">
+      <c r="T4" t="inlineStr">
         <is>
           <t>Specification name (3)</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>Specification value (3)</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>Specification UOM (3)</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="W4" t="inlineStr">
         <is>
           <t>Custom identification name (1)</t>
         </is>
       </c>
-      <c r="W4" t="inlineStr">
+      <c r="X4" t="inlineStr">
         <is>
           <t>Custom identification value (1)</t>
         </is>
       </c>
-      <c r="X4" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>Procurement item</t>
         </is>
       </c>
-      <c r="Y4" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>Procurement item price currency code</t>
         </is>
       </c>
-      <c r="Z4" t="inlineStr">
+      <c r="AA4" t="inlineStr">
         <is>
           <t>Procurement item price</t>
         </is>
       </c>
-      <c r="AA4" t="inlineStr">
+      <c r="AB4" t="inlineStr">
         <is>
           <t>Sales item</t>
         </is>
       </c>
-      <c r="AB4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>Tag (1)</t>
         </is>
       </c>
-      <c r="AC4" t="inlineStr">
+      <c r="AD4" t="inlineStr">
         <is>
           <t>Tag (2)</t>
         </is>
       </c>
-      <c r="AD4" t="inlineStr">
+      <c r="AE4" t="inlineStr">
         <is>
           <t>Tag (3)</t>
         </is>
       </c>
-      <c r="AE4" t="inlineStr">
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>Tag (4)</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
         <is>
           <t>Level</t>
         </is>
       </c>
-      <c r="AF4" t="inlineStr">
+      <c r="AH4" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="AG4" t="inlineStr">
+      <c r="AI4" t="inlineStr">
         <is>
           <t>Base BOM Qty</t>
         </is>
       </c>
-      <c r="AH4" t="inlineStr">
+      <c r="AJ4" t="inlineStr">
         <is>
           <t>Procurement entity name</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
+      <c r="AK4" t="inlineStr">
         <is>
           <t>Preferred vendor code</t>
         </is>
       </c>
-      <c r="AJ4" t="inlineStr">
+      <c r="AL4" t="inlineStr">
         <is>
           <t>Alternate Item Name for Preferred Vendor</t>
         </is>
       </c>
-      <c r="AK4" t="inlineStr">
+      <c r="AM4" t="inlineStr">
         <is>
           <t>Preferred vendor code</t>
         </is>
       </c>
-      <c r="AL4" t="inlineStr">
+      <c r="AN4" t="inlineStr">
         <is>
           <t>Alternate Item Name for Preferred Vendor</t>
         </is>

</xml_diff>